<commit_message>
feat(release): seal controlled demo pipeline evidence and delivery gates
Wire admiral into the DAG, freeze TFL catalog and findings disposition for
non-submission demo scope, and bind full ODA full_dag proof telemetry with
stable run_scope schema so release-run and candidate gates can pass cleanly.
</commit_message>
<xml_diff>
--- a/00_specifications/ADaM_spec.xlsx
+++ b/00_specifications/ADaM_spec.xlsx
@@ -1003,6 +1003,11 @@
           <t>Protocol</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Protocol identifier from study_config.yaml and SDTM study domain records.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1041,6 +1046,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>SDTM.DM.USUBJID.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1079,6 +1089,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>SDTM.DM.SUBJID.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1117,6 +1132,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>SDTM.DM.SITEID.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1155,6 +1175,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>SDTM.DM.AGE.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1198,6 +1223,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Derived age group from SDTM.DM.AGE and protocol age group definitions.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1236,6 +1266,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Numeric age group from AGEGR1.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1274,6 +1309,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>SDTM.DM.RACE.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1312,6 +1352,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>SDTM.DM.ETHNIC.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1355,6 +1400,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>SDTM.DM.SEX.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1398,6 +1448,11 @@
           <t>Assigned</t>
         </is>
       </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Randomized/planned treatment assignment from SDTM.DM.ARM and study_config.yaml treatment map.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1441,6 +1496,11 @@
           <t>Assigned</t>
         </is>
       </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Numeric planned treatment assignment from study_config.yaml treatment map.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1484,6 +1544,11 @@
           <t>Assigned</t>
         </is>
       </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Actual treatment assignment from first non-missing SDTM.EX exposure record and study_config.yaml treatment map.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1527,6 +1592,11 @@
           <t>Assigned</t>
         </is>
       </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Numeric actual treatment assignment from first non-missing SDTM.EX exposure record and study_config.yaml treatment map.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1565,6 +1635,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Randomization date from SDTM.DM.RFSTDTC or randomization source record.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1608,6 +1683,11 @@
           <t>MT.TRTSDT</t>
         </is>
       </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>First exposure start date from SDTM.EX.EXSTDTC.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1651,6 +1731,11 @@
           <t>MT.TRTEDT</t>
         </is>
       </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Last exposure end date from SDTM.EX.EXENDTC.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1694,6 +1779,11 @@
           <t>MT.TRTDURD</t>
         </is>
       </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Derived from ADSL.TRTSDT and ADSL.TRTEDT.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1742,6 +1832,11 @@
           <t>MT.ITTFL</t>
         </is>
       </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Population flag from randomized subject records and protocol population rules.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1790,6 +1885,11 @@
           <t>MT.SAFFL</t>
         </is>
       </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Population flag from treated subject records using SDTM.EX exposure evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1833,6 +1933,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Protocol/per-protocol eligibility source records and protocol deviation review.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1876,6 +1981,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Death flag from SDTM.DM.DTHFL and disposition/death records.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1914,6 +2024,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>MT.DTHDT</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Death date from SDTM.DM.DTHDTC or disposition/death records.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1952,6 +2072,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Death cause from disposition/death source records.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1990,6 +2115,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>MT.LSTALVDT</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Last known alive date from maximum non-death contact/assessment date across SDTM source domains.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2033,6 +2168,11 @@
           <t>MT.ECOGBL</t>
         </is>
       </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Baseline ECOG from SDTM.QS/VS assessment source before treatment start.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2081,6 +2221,11 @@
           <t>MT.MEASDISF</t>
         </is>
       </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Measurable disease flag from baseline tumor/response source assessments.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2124,6 +2269,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Visceral disease flag from baseline lesion source assessments.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2172,6 +2322,11 @@
           <t>MT.PAINBL</t>
         </is>
       </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Baseline pain score from pain assessment source before treatment start.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2210,6 +2365,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Baseline PSA from SDTM.LB prostate-specific antigen records.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2248,6 +2408,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Baseline alkaline phosphatase from SDTM.LB records.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2286,6 +2451,11 @@
           <t>Assigned</t>
         </is>
       </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Baseline albumin from SDTM.LB records.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2324,6 +2494,11 @@
           <t>Assigned</t>
         </is>
       </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Baseline lactate dehydrogenase from SDTM.LB records.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2362,6 +2537,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Baseline hemoglobin from SDTM.LB records.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2400,6 +2580,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Investigator-assessed progression source records.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2443,6 +2628,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Investigator-assessed response source records.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2486,6 +2676,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>MT.ECOGBLIF</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Imputation flag derived from ECOGBL source availability and baseline window rules.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2529,6 +2729,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>MT.PSABLIF</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Imputation flag derived from PSABL source availability and baseline window rules.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2572,6 +2782,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>MT.ALPBLIF</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Imputation flag derived from ALPBL source availability and baseline window rules.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2615,6 +2835,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>MT.HGBBLIF</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Imputation flag derived from HGBBL source availability and baseline window rules.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2658,6 +2888,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>MT.ALBBLIF</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Imputation flag derived from ALBBL source availability and baseline window rules.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2701,6 +2941,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>MT.LDHBLIF</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Imputation flag derived from LDHBL source availability and baseline window rules.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2739,6 +2989,11 @@
           <t>Protocol</t>
         </is>
       </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Protocol identifier from study_config.yaml and SDTM study domain records.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2777,6 +3032,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>SDTM.DM.USUBJID.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2815,6 +3075,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>SDTM.DM.SUBJID.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2858,6 +3123,11 @@
           <t>Assigned</t>
         </is>
       </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Randomized/planned treatment assignment from SDTM.DM.ARM and study_config.yaml treatment map.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2901,6 +3171,11 @@
           <t>Assigned</t>
         </is>
       </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Numeric planned treatment assignment from study_config.yaml treatment map.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2939,6 +3214,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Treatment start date inherited from ADSL.TRTSDT unless defined directly for ADSL.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2982,6 +3262,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Analysis parameter code from dataset-specific parameter derivation and source test/category.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -3020,6 +3305,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Analysis parameter label from dataset-specific parameter derivation and source test/category.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -3058,6 +3348,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Analysis parameter category from dataset-specific parameter map.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -3096,6 +3391,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>MT.ADEX_AVAL</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Numeric exposure analysis value from SDTM.EX dose/duration fields by PARAMCD.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -3134,6 +3439,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>MT.ADEX_AVALC</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Character exposure analysis value from SDTM.EX dose/duration fields by PARAMCD.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -3172,6 +3487,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Analysis visit derived from source visit/date and dataset-specific visit window rules.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -3210,6 +3530,11 @@
           <t>Protocol</t>
         </is>
       </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Protocol identifier from study_config.yaml and SDTM study domain records.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -3248,6 +3573,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>SDTM.DM.USUBJID.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3286,6 +3616,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>SDTM.CM plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -3324,6 +3659,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>SDTM.CM plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -3362,6 +3702,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>SDTM.CM plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -3397,7 +3742,17 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Collected</t>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>MT.ADCM_ASTDT</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>Analysis start date derived from source start date.</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3790,17 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Collected</t>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>MT.ADCM_AENDT</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Analysis end date derived from source end date.</t>
         </is>
       </c>
     </row>
@@ -3476,6 +3841,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>SDTM.CM plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3511,7 +3881,17 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Collected</t>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>MT.ADCM_ASTDY</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>Analysis start relative day derived from ASTDT and ADSL.TRTSDT.</t>
         </is>
       </c>
     </row>
@@ -3557,6 +3937,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>SDTM.CM plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -3600,6 +3985,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>SDTM.CM plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -3643,6 +4033,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>SDTM.CM plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -3681,6 +4076,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>SDTM.CM plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -3724,6 +4124,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>SDTM.CM plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -3767,6 +4172,11 @@
           <t>Assigned</t>
         </is>
       </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>SDTM.CM plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3805,6 +4215,11 @@
           <t>Protocol</t>
         </is>
       </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>Protocol identifier from study_config.yaml and SDTM study domain records.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -3843,6 +4258,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>SDTM.DM.USUBJID.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -3881,6 +4301,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>SDTM.AE/SUPPAE plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3919,6 +4344,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>SDTM.AE/SUPPAE plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3957,6 +4387,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>SDTM.AE/SUPPAE plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -3995,6 +4430,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>SDTM.AE/SUPPAE plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -4033,6 +4473,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>MT.ADAE_ATOXGR</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>Numeric toxicity grade derived from SDTM.AE toxicity grade/severity source fields.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -4076,6 +4526,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>SDTM.AE/SUPPAE plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -4114,6 +4569,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>SDTM.AE/SUPPAE plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -4152,6 +4612,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>Analysis start date derived from source start date.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -4190,6 +4655,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>Analysis end date derived from source end date.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -4228,6 +4698,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>Analysis start relative day derived from ASTDT and ADSL.TRTSDT.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -4266,6 +4741,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>Analysis end relative day derived from AENDT and ADSL.TRTSDT.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -4304,6 +4784,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>SDTM.AE/SUPPAE plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -4342,6 +4827,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>SDTM.AE/SUPPAE plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -4380,6 +4870,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>SDTM.AE/SUPPAE plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -4418,6 +4913,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>SDTM.AE/SUPPAE plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -4456,6 +4956,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>SDTM.AE/SUPPAE plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -4494,6 +4999,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>SDTM.AE/SUPPAE plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -4532,6 +5042,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>SDTM.AE/SUPPAE plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -4570,6 +5085,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>SDTM.AE/SUPPAE plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -4608,6 +5128,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>SDTM.AE/SUPPAE plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -4651,6 +5176,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>SDTM.AE/SUPPAE plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -4694,6 +5224,11 @@
           <t>Assigned</t>
         </is>
       </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>Treatment-emergent flag derived from ADAE.ASTDT and ADSL.TRTSDT.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -4732,6 +5267,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>Adverse event duration derived from ADAE.ASTDT and ADAE.AENDT.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -4770,6 +5310,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>Duration unit assigned by adverse-event derivation rule.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -4808,6 +5353,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>SDTM.AE/SUPPAE plus ADSL treatment and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -4851,6 +5401,11 @@
           <t>Assigned</t>
         </is>
       </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>Actual treatment assignment inherited from ADSL.TRT01A.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -4894,6 +5449,11 @@
           <t>Assigned</t>
         </is>
       </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>Numeric actual treatment assignment inherited from ADSL.TRT01AN.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -4932,6 +5492,11 @@
           <t>Protocol</t>
         </is>
       </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>Protocol identifier from study_config.yaml and SDTM study domain records.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -4970,6 +5535,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>SDTM.DM.USUBJID.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -5008,6 +5578,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>SDTM.DM.SUBJID.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -5051,6 +5626,11 @@
           <t>Assigned</t>
         </is>
       </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>Randomized/planned treatment assignment from SDTM.DM.ARM and study_config.yaml treatment map.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -5089,6 +5669,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>Treatment start date inherited from ADSL.TRTSDT unless defined directly for ADSL.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -5132,6 +5717,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>Analysis parameter code from dataset-specific parameter derivation and source test/category.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -5170,6 +5760,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>Analysis parameter label from dataset-specific parameter derivation and source test/category.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -5208,6 +5803,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>Numeric parameter ordering from dataset-specific parameter map.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -5246,6 +5846,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>Analysis parameter category from dataset-specific parameter map.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -5284,6 +5889,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>MT.ADLB_AVAL</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>Numeric lab analysis value from SDTM.LB.LBSTRESN.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -5322,6 +5937,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>MT.ADLB_AVALC</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>Character lab analysis value from SDTM.LB.LBSTRESC.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -5360,6 +5985,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>SDTM.LB plus ADSL treatment, baseline, and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -5398,6 +6028,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>SDTM.LB plus ADSL treatment, baseline, and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -5436,6 +6071,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>SDTM.LB plus ADSL treatment, baseline, and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -5474,6 +6114,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>Analysis visit derived from source visit/date and dataset-specific visit window rules.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -5512,6 +6157,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>Numeric analysis visit derived from AVISIT and dataset-specific visit ordering.</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -5550,6 +6200,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>SDTM.LB plus ADSL treatment, baseline, and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -5588,6 +6243,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>MT.ADLB_ATOXGR</t>
+        </is>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>Analysis toxicity grade derived from SDTM.LB result, normal range, and grading rules.</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -5626,6 +6291,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>MT.ADLB_BASE</t>
+        </is>
+      </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>Baseline numeric value selected from pre-treatment ADLB.AVAL records.</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -5664,6 +6339,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>MT.ADLB_BASEC</t>
+        </is>
+      </c>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>Baseline character value selected from pre-treatment ADLB.AVALC records.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -5702,6 +6387,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>Baseline toxicity grade selected from pre-treatment records.</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -5740,6 +6430,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>MT.ADLB_CHG</t>
+        </is>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>Change from baseline derived as ADLB.AVAL minus ADLB.BASE.</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -5778,6 +6478,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>MT.ADLB_PCHG</t>
+        </is>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>Percent change from baseline derived as ADLB.CHG divided by ADLB.BASE.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -5821,6 +6531,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>Analysis inclusion flag derived from dataset-specific record-selection rules.</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -5864,6 +6579,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>MT.ADLB_BASEFL</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>Baseline flag derived from pre-treatment record-selection rules.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -5902,6 +6627,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>SDTM.LB plus ADSL treatment, baseline, and subject-level attributes.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -5940,6 +6670,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>MT.ADLB_ADT</t>
+        </is>
+      </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>Analysis date from SDTM.LB.LBDTC.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -5978,6 +6718,11 @@
           <t>Protocol</t>
         </is>
       </c>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>Protocol identifier from study_config.yaml and SDTM study domain records.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -6016,6 +6761,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>SDTM.DM.USUBJID.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -6054,6 +6804,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>SDTM.DM.SUBJID.</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -6097,6 +6852,11 @@
           <t>Assigned</t>
         </is>
       </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>Randomized/planned treatment assignment from SDTM.DM.ARM and study_config.yaml treatment map.</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -6135,6 +6895,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>Treatment start date inherited from ADSL.TRTSDT unless defined directly for ADSL.</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -6178,6 +6943,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>Analysis parameter code from dataset-specific parameter derivation and source test/category.</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -6216,6 +6986,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t>Analysis parameter label from dataset-specific parameter derivation and source test/category.</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -6254,6 +7029,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>MT.ADRS_AVALC</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>Character response result from response source assessments and response derivation rules.</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -6292,6 +7077,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>Analysis date derived from the source assessment date.</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -6330,6 +7120,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>Analysis relative day derived from ADT and ADSL.TRTSDT.</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -6368,6 +7163,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>Analysis visit derived from source visit/date and dataset-specific visit window rules.</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -6411,6 +7211,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>Analysis inclusion flag derived from dataset-specific record-selection rules.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -6449,6 +7254,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>MT.ADRS_AVAL</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>Numeric response category from ADRS.AVALC response ordering map.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -6487,6 +7302,11 @@
           <t>Protocol</t>
         </is>
       </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>Protocol identifier from study_config.yaml and SDTM study domain records.</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -6525,6 +7345,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>SDTM.DM.USUBJID.</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -6563,6 +7388,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>SDTM.DM.SUBJID.</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -6601,6 +7431,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>SDTM.DM.SITEID.</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -6644,6 +7479,11 @@
           <t>Assigned</t>
         </is>
       </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>Randomized/planned treatment assignment from SDTM.DM.ARM and study_config.yaml treatment map.</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -6687,6 +7527,11 @@
           <t>Assigned</t>
         </is>
       </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>Numeric planned treatment assignment from study_config.yaml treatment map.</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -6730,6 +7575,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>MT.ADTTE_ITTFL</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>Inherited from ADSL.ITTFL.</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -6773,6 +7628,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>MT.ADTTE_SAFFL</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>Inherited from ADSL.SAFFL.</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -6816,6 +7681,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>Analysis parameter code from dataset-specific parameter derivation and source test/category.</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -6854,6 +7724,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>Analysis parameter label from dataset-specific parameter derivation and source test/category.</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -6892,6 +7767,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>MT.ADTTE_PARAMN</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>Numeric parameter ordering from ADTTE.PARAMCD.</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -6930,6 +7815,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>MT.ADTTE_PARCAT1</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>Time-to-event category from ADTTE.PARAMCD.</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -6968,6 +7863,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>ADSL subject-level attributes plus SDTM.DS, SDTM.RS/LS, SDTM.AE, and death/progression source dates by PARAMCD.</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -7006,6 +7906,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>Analysis date derived from the source assessment date.</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -7054,6 +7959,11 @@
           <t>MT.CNSR_TTE</t>
         </is>
       </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>Censoring indicator derived from event/censor source dates by ADTTE.PARAMCD.</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -7092,6 +8002,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>ADSL subject-level attributes plus SDTM.DS, SDTM.RS/LS, SDTM.AE, and death/progression source dates by PARAMCD.</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -7130,6 +8045,11 @@
           <t>Collected</t>
         </is>
       </c>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>ADSL subject-level attributes plus SDTM.DS, SDTM.RS/LS, SDTM.AE, and death/progression source dates by PARAMCD.</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -7173,6 +8093,11 @@
           <t>MT.AVAL_TTE</t>
         </is>
       </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>Time-to-event duration derived from ADTTE.STARTDT, ADTTE.ADT, and ADTTE.AVALU.</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -7211,6 +8136,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>MT.ADTTE_AVALU</t>
+        </is>
+      </c>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>Time-to-event unit assigned by ADTTE parameter derivation.</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -7249,6 +8184,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>MT.ADEX_PARAMN</t>
+        </is>
+      </c>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>Numeric parameter ordering from ADEX.PARAMCD.</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -7285,6 +8230,16 @@
       <c r="K160" t="inlineStr">
         <is>
           <t>Derived</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>MT.ADEX_AVISITN</t>
+        </is>
+      </c>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>Numeric analysis visit derived from ADEX.AVISIT and SDTM.EX sequence/date.</t>
         </is>
       </c>
     </row>
@@ -9944,7 +10899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" customFormat="1" s="1">
@@ -10294,6 +11249,710 @@
       <c r="D15" t="inlineStr">
         <is>
           <t>Censoring indicator, set to 0 if the event occurred, or 1 if censored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MT.DTHDT</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Method for DTHDT</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Death date derived from SDTM.DM.DTHDTC or disposition/death records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MT.LSTALVDT</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Method for LSTALVDT</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Last known alive date derived as the maximum non-death contact or assessment date across source domains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>MT.ECOGBLIF</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Method for ECOGBLIF</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Baseline ECOG imputation flag derived from ECOGBL source availability and baseline window rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>MT.PSABLIF</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Method for PSABLIF</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Baseline PSA imputation flag derived from PSABL source availability and baseline window rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>MT.ALPBLIF</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Method for ALPBLIF</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Baseline alkaline phosphatase imputation flag derived from ALPBL source availability and baseline window rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>MT.HGBBLIF</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Method for HGBBLIF</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Baseline hemoglobin imputation flag derived from HGBBL source availability and baseline window rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>MT.ALBBLIF</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Method for ALBBLIF</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Baseline albumin imputation flag derived from ALBBL source availability and baseline window rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>MT.LDHBLIF</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Method for LDHBLIF</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Baseline lactate dehydrogenase imputation flag derived from LDHBL source availability and baseline window rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>MT.ADEX_AVAL</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Method for ADEX_AVAL</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Numeric exposure analysis value derived from SDTM.EX dose, duration, or cycle records according to ADEX.PARAMCD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>MT.ADEX_AVALC</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Method for ADEX_AVALC</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Character exposure analysis value derived from SDTM.EX dose, duration, or cycle records according to ADEX.PARAMCD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MT.ADEX_PARAMN</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Method for ADEX_PARAMN</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Numeric ADEX parameter ordering derived from ADEX.PARAMCD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MT.ADEX_AVISITN</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Method for ADEX_AVISITN</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Numeric ADEX analysis visit derived from ADEX.AVISIT and SDTM.EX date or sequence ordering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>MT.ADAE_ATOXGR</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Method for ADAE_ATOXGR</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Numeric adverse-event toxicity grade derived from SDTM.AE toxicity grade or severity source fields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>MT.ADLB_AVAL</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Method for ADLB_AVAL</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Numeric laboratory analysis value derived from SDTM.LB.LBSTRESN after parameter-specific unit standardization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>MT.ADLB_AVALC</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Method for ADLB_AVALC</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Character laboratory analysis value derived from SDTM.LB.LBSTRESC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>MT.ADLB_ATOXGR</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Method for ADLB_ATOXGR</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Analysis toxicity grade derived from laboratory result, normal range, and grading rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>MT.ADLB_BASE</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Method for ADLB_BASE</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Baseline numeric value selected from the latest eligible pre-treatment ADLB.AVAL record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>MT.ADLB_BASEC</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Method for ADLB_BASEC</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Baseline character value selected from the latest eligible pre-treatment ADLB.AVALC record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>MT.ADLB_CHG</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Method for ADLB_CHG</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Change from baseline calculated as ADLB.AVAL minus ADLB.BASE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>MT.ADLB_PCHG</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Method for ADLB_PCHG</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Percent change from baseline calculated as 100 times ADLB.CHG divided by ADLB.BASE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>MT.ADLB_BASEFL</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Method for ADLB_BASEFL</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Baseline flag set on the selected eligible pre-treatment laboratory record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>MT.ADLB_ADT</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Method for ADLB_ADT</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Analysis date derived from SDTM.LB.LBDTC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>MT.ADRS_AVALC</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Method for ADRS_AVALC</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Character response result derived from response source assessments and response derivation rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>MT.ADRS_AVAL</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Method for ADRS_AVAL</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Numeric response category derived from ADRS.AVALC response ordering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>MT.ADTTE_ITTFL</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Method for ADTTE_ITTFL</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Intent-to-treat flag inherited from ADSL.ITTFL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>MT.ADTTE_SAFFL</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Method for ADTTE_SAFFL</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Safety population flag inherited from ADSL.SAFFL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>MT.ADTTE_PARAMN</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Method for ADTTE_PARAMN</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Numeric ADTTE parameter ordering derived from ADTTE.PARAMCD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>MT.ADTTE_PARCAT1</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Method for ADTTE_PARCAT1</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Time-to-event parameter category derived from ADTTE.PARAMCD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>MT.ADTTE_AVALU</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Method for ADTTE_AVALU</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Time-to-event unit assigned by ADTTE parameter derivation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>MT.ADCM_ASTDT</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Method for ADCM_ASTDT</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Analysis medication start date derived from SDTM.CM.CMSTDTC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>MT.ADCM_AENDT</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Method for ADCM_AENDT</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Analysis medication end date derived from SDTM.CM.CMENDTC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>MT.ADCM_ASTDY</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Method for ADCM_ASTDY</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Computation</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Analysis medication start relative day derived from ADCM.ASTDT and ADSL.TRTSDT.</t>
         </is>
       </c>
     </row>

</xml_diff>